<commit_message>
fix(back-end): fix get valid product
</commit_message>
<xml_diff>
--- a/src/services/data/interaction_scores.xlsx
+++ b/src/services/data/interaction_scores.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,13 +418,13 @@
         <v>6739a4c617dc7ef140b34295</v>
       </c>
       <c r="B2" t="str">
-        <v>6728f96acb86d3695fa1f4a6</v>
+        <v>6728e9cd071b8fcf4f501df9</v>
       </c>
       <c r="C2">
-        <v>0.7</v>
+        <v>0.9182</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-14T14:55:57.539Z</v>
       </c>
     </row>
     <row r="3">
@@ -432,13 +432,13 @@
         <v>6739a4c617dc7ef140b34295</v>
       </c>
       <c r="B3" t="str">
-        <v>6728e8a8071b8fcf4f501df0</v>
+        <v>6728ea18071b8fcf4f501dff</v>
       </c>
       <c r="C3">
-        <v>0.7</v>
+        <v>0.7818</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-02-12T11:31:56.846Z</v>
+        <v>2025-06-14T14:56:59.434Z</v>
       </c>
     </row>
     <row r="4">
@@ -446,13 +446,13 @@
         <v>6739a4c617dc7ef140b34295</v>
       </c>
       <c r="B4" t="str">
-        <v>6728e9ab071b8fcf4f501df6</v>
+        <v>68067520286f80e4174d8723</v>
       </c>
       <c r="C4">
-        <v>0.88</v>
+        <v>0.0273</v>
       </c>
       <c r="D4" t="str">
-        <v>2025-04-13T11:31:56.846Z</v>
+        <v>2025-06-14T12:55:31.370Z</v>
       </c>
     </row>
     <row r="5">
@@ -460,125 +460,125 @@
         <v>6739a4c617dc7ef140b34295</v>
       </c>
       <c r="B5" t="str">
-        <v>6728e9e6071b8fcf4f501dfc</v>
+        <v>6728e93a071b8fcf4f501df3</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="D5" t="str">
-        <v>2025-06-07T03:28:32.552Z</v>
+        <v>2025-06-14T14:27:32.204Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B6" t="str">
-        <v>6728ea62071b8fcf4f501e02</v>
+        <v>6728f96acb86d3695fa1f4a6</v>
       </c>
       <c r="C6">
         <v>0.82</v>
       </c>
       <c r="D6" t="str">
-        <v>2025-04-13T11:31:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B7" t="str">
-        <v>6743a3a8fd3ceed5b16a5e18</v>
+        <v>676137906c06138b1419f8a5</v>
       </c>
       <c r="C7">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
       <c r="D7" t="str">
-        <v>2025-04-13T11:31:56.846Z</v>
+        <v>2025-02-20T10:25:56.846Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B8" t="str">
-        <v>676137906c06138b1419f8a5</v>
+        <v>676137906c06138b1419f8a6</v>
       </c>
       <c r="C8">
-        <v>0.94</v>
+        <v>1</v>
       </c>
       <c r="D8" t="str">
-        <v>2025-04-13T11:31:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B9" t="str">
-        <v>67f08cab1841d535b6af6f50</v>
+        <v>67f08dde1841d535b6af6f5e</v>
       </c>
       <c r="C9">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="D9" t="str">
-        <v>2025-04-13T11:31:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B10" t="str">
-        <v>67f08e231841d535b6af6f67</v>
+        <v>67f08ef11841d535b6af6f6f</v>
       </c>
       <c r="C10">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-04-13T11:31:56.846Z</v>
+        <v>2025-02-20T10:25:56.846Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B11" t="str">
-        <v>6728eb4a071b8fcf4f501e0b</v>
+        <v>67f090e61841d535b6af6f78</v>
       </c>
       <c r="C11">
-        <v>0.76</v>
+        <v>0.7</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-05-23T04:46:31.245Z</v>
+        <v>2025-02-20T10:25:56.846Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B12" t="str">
-        <v>6728e93a071b8fcf4f501df3</v>
+        <v>67f091181841d535b6af6f7b</v>
       </c>
       <c r="C12">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-02-20T10:25:56.846Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>6739a4c617dc7ef140b34295</v>
+        <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B13" t="str">
-        <v>6728eac6071b8fcf4f501e05</v>
+        <v>67f091da1841d535b6af6f7e</v>
       </c>
       <c r="C13">
-        <v>0.06</v>
+        <v>0.7</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-02-20T10:25:56.846Z</v>
       </c>
     </row>
     <row r="14">
@@ -586,13 +586,13 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B14" t="str">
-        <v>6728f96acb86d3695fa1f4a6</v>
+        <v>67f092ce1841d535b6af6f84</v>
       </c>
       <c r="C14">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-02-20T10:25:56.846Z</v>
       </c>
     </row>
     <row r="15">
@@ -600,7 +600,7 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B15" t="str">
-        <v>676137906c06138b1419f8a5</v>
+        <v>67f093171841d535b6af6f8a</v>
       </c>
       <c r="C15">
         <v>0.7</v>
@@ -614,10 +614,10 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B16" t="str">
-        <v>676137906c06138b1419f8a6</v>
+        <v>67f08d651841d535b6af6f57</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0.03</v>
       </c>
       <c r="D16" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -628,10 +628,10 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B17" t="str">
-        <v>67f08dde1841d535b6af6f5e</v>
+        <v>6728e9e6071b8fcf4f501dfc</v>
       </c>
       <c r="C17">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="D17" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -642,13 +642,13 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B18" t="str">
-        <v>67f08ef11841d535b6af6f6f</v>
+        <v>6728ea62071b8fcf4f501e02</v>
       </c>
       <c r="C18">
-        <v>0.7</v>
+        <v>0.18</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-02-20T10:25:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="19">
@@ -656,13 +656,13 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B19" t="str">
-        <v>67f090e61841d535b6af6f78</v>
+        <v>6728eac6071b8fcf4f501e05</v>
       </c>
       <c r="C19">
-        <v>0.7</v>
+        <v>0.09</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-02-20T10:25:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="20">
@@ -670,13 +670,13 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B20" t="str">
-        <v>67f091181841d535b6af6f7b</v>
+        <v>6728ebbb071b8fcf4f501e11</v>
       </c>
       <c r="C20">
-        <v>0.7</v>
+        <v>0.27</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-02-20T10:25:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="21">
@@ -684,13 +684,13 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B21" t="str">
-        <v>67f091da1841d535b6af6f7e</v>
+        <v>6728ec07071b8fcf4f501e17</v>
       </c>
       <c r="C21">
-        <v>0.7</v>
+        <v>0.12</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-02-20T10:25:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="22">
@@ -698,38 +698,38 @@
         <v>67236aac181cccce457a7489</v>
       </c>
       <c r="B22" t="str">
-        <v>67f092ce1841d535b6af6f84</v>
+        <v>67447fbced2b056beb0f8e01</v>
       </c>
       <c r="C22">
-        <v>0.7</v>
+        <v>0.24</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-02-20T10:25:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B23" t="str">
-        <v>67f093171841d535b6af6f8a</v>
+        <v>67447fbced2b056beb0f8e01</v>
       </c>
       <c r="C23">
         <v>0.7</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-02-20T10:25:56.846Z</v>
+        <v>2025-03-12T11:31:56.846Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B24" t="str">
-        <v>67f08d651841d535b6af6f57</v>
+        <v>676137906c06138b1419f8a5</v>
       </c>
       <c r="C24">
-        <v>0.03</v>
+        <v>0.7</v>
       </c>
       <c r="D24" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -737,13 +737,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B25" t="str">
-        <v>6728e9e6071b8fcf4f501dfc</v>
+        <v>67f08d651841d535b6af6f57</v>
       </c>
       <c r="C25">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D25" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -751,13 +751,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B26" t="str">
-        <v>6728ea62071b8fcf4f501e02</v>
+        <v>6728ebbb071b8fcf4f501e11</v>
       </c>
       <c r="C26">
-        <v>0.18</v>
+        <v>0.7</v>
       </c>
       <c r="D26" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -765,13 +765,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B27" t="str">
-        <v>6728eac6071b8fcf4f501e05</v>
+        <v>6728ea62071b8fcf4f501e02</v>
       </c>
       <c r="C27">
-        <v>0.09</v>
+        <v>0.7</v>
       </c>
       <c r="D27" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -779,13 +779,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B28" t="str">
-        <v>6728ebbb071b8fcf4f501e11</v>
+        <v>6728e9ab071b8fcf4f501df6</v>
       </c>
       <c r="C28">
-        <v>0.27</v>
+        <v>0.7</v>
       </c>
       <c r="D28" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -793,13 +793,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B29" t="str">
-        <v>6728ec07071b8fcf4f501e17</v>
+        <v>67250625bb931ab886fc69db</v>
       </c>
       <c r="C29">
-        <v>0.12</v>
+        <v>0.7</v>
       </c>
       <c r="D29" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -807,13 +807,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>67236aac181cccce457a7489</v>
+        <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B30" t="str">
-        <v>67447fbced2b056beb0f8e01</v>
+        <v>6728ea18071b8fcf4f501dff</v>
       </c>
       <c r="C30">
-        <v>0.24</v>
+        <v>0.7</v>
       </c>
       <c r="D30" t="str">
         <v>2025-03-12T11:31:56.846Z</v>
@@ -824,13 +824,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B31" t="str">
-        <v>67447fbced2b056beb0f8e01</v>
+        <v>6728eac6071b8fcf4f501e05</v>
       </c>
       <c r="C31">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-08T08:04:41.421Z</v>
       </c>
     </row>
     <row r="32">
@@ -838,13 +838,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B32" t="str">
-        <v>676137906c06138b1419f8a5</v>
+        <v>6728e9cd071b8fcf4f501df9</v>
       </c>
       <c r="C32">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-12T08:21:14.626Z</v>
       </c>
     </row>
     <row r="33">
@@ -852,13 +852,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B33" t="str">
-        <v>67f08d651841d535b6af6f57</v>
+        <v>67f094111841d535b6af6f99</v>
       </c>
       <c r="C33">
-        <v>0.7</v>
+        <v>0.05</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-01T05:27:27.719Z</v>
       </c>
     </row>
     <row r="34">
@@ -866,13 +866,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B34" t="str">
-        <v>6728ebbb071b8fcf4f501e11</v>
+        <v>67f092321841d535b6af6f81</v>
       </c>
       <c r="C34">
-        <v>0.7</v>
+        <v>0.15</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-01T05:45:55.487Z</v>
       </c>
     </row>
     <row r="35">
@@ -880,13 +880,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B35" t="str">
-        <v>6728ea62071b8fcf4f501e02</v>
+        <v>6728e8a8071b8fcf4f501df0</v>
       </c>
       <c r="C35">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-01T07:32:49.957Z</v>
       </c>
     </row>
     <row r="36">
@@ -894,13 +894,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B36" t="str">
-        <v>6728e9ab071b8fcf4f501df6</v>
+        <v>67f095371841d535b6af6fb1</v>
       </c>
       <c r="C36">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-01T07:48:03.296Z</v>
       </c>
     </row>
     <row r="37">
@@ -908,13 +908,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B37" t="str">
-        <v>67250625bb931ab886fc69db</v>
+        <v>6728ec07071b8fcf4f501e17</v>
       </c>
       <c r="C37">
-        <v>0.7</v>
+        <v>0.05</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-01T07:57:47.828Z</v>
       </c>
     </row>
     <row r="38">
@@ -922,13 +922,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B38" t="str">
-        <v>6728e9e6071b8fcf4f501dfc</v>
+        <v>6728ebe1071b8fcf4f501e14</v>
       </c>
       <c r="C38">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-06-06T08:18:39.769Z</v>
+        <v>2025-06-08T16:12:13.945Z</v>
       </c>
     </row>
     <row r="39">
@@ -936,13 +936,13 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B39" t="str">
-        <v>6728ea18071b8fcf4f501dff</v>
+        <v>6728f96acb86d3695fa1f4a6</v>
       </c>
       <c r="C39">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-08T07:54:50.190Z</v>
       </c>
     </row>
     <row r="40">
@@ -950,298 +950,172 @@
         <v>6738b019504ed0629a25b8b1</v>
       </c>
       <c r="B40" t="str">
-        <v>6728eac6071b8fcf4f501e05</v>
+        <v>6728e9e6071b8fcf4f501dfc</v>
       </c>
       <c r="C40">
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-03-12T11:31:56.846Z</v>
+        <v>2025-06-12T08:20:59.446Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B41" t="str">
-        <v>6728e9cd071b8fcf4f501df9</v>
+        <v>6728e9e6071b8fcf4f501dfc</v>
       </c>
       <c r="C41">
-        <v>0.3</v>
+        <v>0.925</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-06-02T05:03:23.943Z</v>
+        <v>2025-05-23T04:41:14.096Z</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B42" t="str">
-        <v>67f095dc1841d535b6af6fba</v>
+        <v>6728e93a071b8fcf4f501df3</v>
       </c>
       <c r="C42">
-        <v>0.075</v>
+        <v>0.775</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-06-01T05:24:22.234Z</v>
+        <v>2025-05-23T09:19:25.598Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B43" t="str">
-        <v>67f094111841d535b6af6f99</v>
+        <v>6728ea18071b8fcf4f501dff</v>
       </c>
       <c r="C43">
-        <v>0.075</v>
+        <v>0.775</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-06-01T05:27:27.719Z</v>
+        <v>2025-05-23T09:19:36.004Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B44" t="str">
-        <v>67f092321841d535b6af6f81</v>
+        <v>67f091181841d535b6af6f7b</v>
       </c>
       <c r="C44">
-        <v>0.225</v>
+        <v>0.775</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-06-01T05:45:55.487Z</v>
+        <v>2025-05-23T09:19:59.350Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B45" t="str">
-        <v>6728e8a8071b8fcf4f501df0</v>
+        <v>6728e9cd071b8fcf4f501df9</v>
       </c>
       <c r="C45">
-        <v>0.15</v>
+        <v>0.925</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-06-01T07:32:49.957Z</v>
+        <v>2025-05-23T09:21:52.485Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B46" t="str">
-        <v>67f095371841d535b6af6fb1</v>
+        <v>6728f96acb86d3695fa1f4a6</v>
       </c>
       <c r="C46">
-        <v>0.3</v>
+        <v>0.775</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-06-01T07:48:03.296Z</v>
+        <v>2025-05-23T09:21:00.865Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>682326702fff19d415752f01</v>
       </c>
       <c r="B47" t="str">
-        <v>6728ec07071b8fcf4f501e17</v>
+        <v>68067dd1286f80e4174d8736</v>
       </c>
       <c r="C47">
-        <v>0.075</v>
+        <v>1</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-06-01T07:57:47.828Z</v>
+        <v>2025-05-23T09:23:22.245Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>683b37622eb85e2df9802771</v>
       </c>
       <c r="B48" t="str">
-        <v>6728ebe1071b8fcf4f501e14</v>
+        <v>6728e93a071b8fcf4f501df3</v>
       </c>
       <c r="C48">
-        <v>0.225</v>
+        <v>1</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-06-02T01:19:45.553Z</v>
+        <v>2025-05-31T17:08:32.178Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>6738b019504ed0629a25b8b1</v>
+        <v>683b37622eb85e2df9802771</v>
       </c>
       <c r="B49" t="str">
-        <v>6728f96acb86d3695fa1f4a6</v>
+        <v>6728ea18071b8fcf4f501dff</v>
       </c>
       <c r="C49">
-        <v>0.075</v>
+        <v>0.85</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-06-04T07:18:47.050Z</v>
+        <v>2025-05-31T17:10:43.229Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>682326702fff19d415752f01</v>
+        <v>683b37622eb85e2df9802771</v>
       </c>
       <c r="B50" t="str">
-        <v>6728e9e6071b8fcf4f501dfc</v>
+        <v>6728f96acb86d3695fa1f4a6</v>
       </c>
       <c r="C50">
-        <v>0.925</v>
+        <v>0.15</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-05-23T04:41:14.096Z</v>
+        <v>2025-06-01T02:53:50.928Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>682326702fff19d415752f01</v>
+        <v>683b37622eb85e2df9802771</v>
       </c>
       <c r="B51" t="str">
-        <v>6728e93a071b8fcf4f501df3</v>
+        <v>6728ec07071b8fcf4f501e17</v>
       </c>
       <c r="C51">
-        <v>0.775</v>
+        <v>0.15</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-05-23T09:19:25.598Z</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>682326702fff19d415752f01</v>
-      </c>
-      <c r="B52" t="str">
-        <v>6728ea18071b8fcf4f501dff</v>
-      </c>
-      <c r="C52">
-        <v>0.775</v>
-      </c>
-      <c r="D52" t="str">
-        <v>2025-05-23T09:19:36.004Z</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>682326702fff19d415752f01</v>
-      </c>
-      <c r="B53" t="str">
-        <v>67f091181841d535b6af6f7b</v>
-      </c>
-      <c r="C53">
-        <v>0.775</v>
-      </c>
-      <c r="D53" t="str">
-        <v>2025-05-23T09:19:59.350Z</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>682326702fff19d415752f01</v>
-      </c>
-      <c r="B54" t="str">
-        <v>6728e9cd071b8fcf4f501df9</v>
-      </c>
-      <c r="C54">
-        <v>0.925</v>
-      </c>
-      <c r="D54" t="str">
-        <v>2025-05-23T09:21:52.485Z</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>682326702fff19d415752f01</v>
-      </c>
-      <c r="B55" t="str">
-        <v>6728f96acb86d3695fa1f4a6</v>
-      </c>
-      <c r="C55">
-        <v>0.775</v>
-      </c>
-      <c r="D55" t="str">
-        <v>2025-05-23T09:21:00.865Z</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>682326702fff19d415752f01</v>
-      </c>
-      <c r="B56" t="str">
-        <v>68067dd1286f80e4174d8736</v>
-      </c>
-      <c r="C56">
-        <v>1</v>
-      </c>
-      <c r="D56" t="str">
-        <v>2025-05-23T09:23:22.245Z</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>683b37622eb85e2df9802771</v>
-      </c>
-      <c r="B57" t="str">
-        <v>6728e93a071b8fcf4f501df3</v>
-      </c>
-      <c r="C57">
-        <v>1</v>
-      </c>
-      <c r="D57" t="str">
-        <v>2025-05-31T17:08:32.178Z</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>683b37622eb85e2df9802771</v>
-      </c>
-      <c r="B58" t="str">
-        <v>6728ea18071b8fcf4f501dff</v>
-      </c>
-      <c r="C58">
-        <v>0.85</v>
-      </c>
-      <c r="D58" t="str">
-        <v>2025-05-31T17:10:43.229Z</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>683b37622eb85e2df9802771</v>
-      </c>
-      <c r="B59" t="str">
-        <v>6728f96acb86d3695fa1f4a6</v>
-      </c>
-      <c r="C59">
-        <v>0.15</v>
-      </c>
-      <c r="D59" t="str">
-        <v>2025-06-01T02:53:50.928Z</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>683b37622eb85e2df9802771</v>
-      </c>
-      <c r="B60" t="str">
-        <v>6728ec07071b8fcf4f501e17</v>
-      </c>
-      <c r="C60">
-        <v>0.15</v>
-      </c>
-      <c r="D60" t="str">
         <v>2025-06-01T07:31:20.015Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>